<commit_message>
Add format/protection to eval sheets; update 楊玉鳳 and 鍾欣芳
- Add apply_format_and_protection(): enables worksheet protection,
  unlocks input cells, extends SUM/IF formulas per evaluatee column,
  updates C5 COUNTIF range
- Regenerate 楊玉鳳 and 鍾欣芳 with correct formulas and cell protection

https://claude.ai/code/session_01P9kqGzeEo3GNvL8KsQpiLU
</commit_message>
<xml_diff>
--- a/eval_output/加工組_張舒涵_評分表.xlsx
+++ b/eval_output/加工組_張舒涵_評分表.xlsx
@@ -130,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -157,6 +157,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -168,6 +171,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -608,7 +615,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>COUNTIF(D6:P6,"&lt;&gt;")</f>
+        <f>COUNTIF(D6:G6,"&lt;&gt;")</f>
         <v/>
       </c>
     </row>
@@ -680,14 +687,18 @@
 ✓不熟悉製程；錯誤率高；無法獨立作業或教導他人。(0-2) </t>
         </is>
       </c>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
     </row>
     <row r="9" ht="84" customHeight="1">
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>產品知識與設備保養管理（10 分）</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">✓熟知產品規格、品質要求、主要不良模式；保養確實、設備狀況佳。 (9-10) 
 ✓了解基本產品要求；保養紀錄完整；偶需提醒。 (7-8) 
@@ -696,6 +707,10 @@
 ✓不不懂產品、不做保養；設備狀況差，影響產線運作。(0-2) </t>
         </is>
       </c>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
     </row>
     <row r="10" ht="53" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -703,12 +718,12 @@
           <t>團隊溝通協調能力20%</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>受評者的溝通協調與配合度</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>✓非常願意溝通協調且配合度極高 (16-20)
 ✓願意溝通協調且配合度高 (12-15)
@@ -717,15 +732,19 @@
 ✓非常不願意溝通協調且配合度極低 (0-3)</t>
         </is>
       </c>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
     </row>
     <row r="11" ht="53" customHeight="1">
       <c r="A11" s="8" t="n"/>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>【現場】「只限評分現場人員專用」</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">✓積極配合排班與加班，並能準時高品質完成工作 (18-20)
 ✓配合加班完成工作，偶有延遲但能解釋清楚且態度積極(14-17)
@@ -736,28 +755,35 @@
 </t>
         </is>
       </c>
-      <c r="D11" s="6" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12" ht="53" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>工作態度
 30%</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>*低於等於3分或高於等於18分，請說明原因：___________________________</t>
         </is>
       </c>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13" ht="105" customHeight="1">
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>受評者在本次受評區間，對於協辦的工作，『完成度』達</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>10分100%
 9分  90%
@@ -771,15 +797,19 @@
 1分  10%</t>
         </is>
       </c>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14" ht="43.5" customHeight="1">
       <c r="A14" s="8" t="n"/>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>※印象中你對受評者在指導與覆核部屬方面，願意給幾分</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">✓經常主動指導(領導)部屬 (16-20)
 ✓需經部屬提出並樂意指導(領導) (11-15)
@@ -788,28 +818,35 @@
 </t>
         </is>
       </c>
-      <c r="D14" s="6" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15" ht="58.5" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>領導統御
 30%</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>*低於等於6分或高於等於16分，請說明原因：________________</t>
         </is>
       </c>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16" ht="49" customHeight="1">
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>是否願意和受評者一起工作?</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>✓我很願意跟受評者一起工作(8~10)
 ✓我還算願意跟受評者一起工作(5~7)
@@ -817,24 +854,43 @@
 ✓我不願意跟受評者一起工作(0-1)</t>
         </is>
       </c>
-      <c r="D16" s="6" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17" ht="29" customHeight="1">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>*低於等於3分或最高分，請敘述狀況：_________________________</t>
         </is>
       </c>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18" ht="50.5" customHeight="1">
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>總分</t>
         </is>
       </c>
-      <c r="D18" s="19">
+      <c r="D18" s="21">
         <f>SUM(D8:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="21">
+        <f>SUM(E8:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="21">
+        <f>SUM(F8:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="21">
+        <f>SUM(G8:G17)</f>
         <v/>
       </c>
     </row>
@@ -849,8 +905,39 @@
 ), "⚠ 超標！", "")</f>
         <v/>
       </c>
+      <c r="E19" s="6">
+        <f>IF(OR(
+  AND(E18&gt;=90, COUNTIF($D$18:$Z$18, "&gt;=90")/COUNTA($D$18:$Z$18)&gt;0.05),
+  AND(E18&gt;=80,E18&lt;=89, (COUNTIF($D$18:$Z$18, "&gt;=80")-COUNTIF($D$18:$Z$18, "&gt;=90"))/COUNTA($D$18:$Z$18)&gt;0.2),
+  AND(E18&gt;=70,E18&lt;=79, (COUNTIF($D$18:$Z$18, "&gt;=70")-COUNTIF($D$18:$Z$18, "&gt;=80"))/COUNTA($D$18:$Z$18)&gt;0.4),
+  AND(E18&gt;=60,E18&lt;=69, (COUNTIF($D$18:$Z$18, "&gt;=60")-COUNTIF($D$18:$Z$18, "&gt;=70"))/COUNTA($D$18:$Z$18)&gt;0.3),
+  AND(E18&lt;=59, COUNTIF($D$18:$Z$18, "&lt;=59")/COUNTA($D$18:$Z$18)&gt;0.05)
+), "⚠ 超標！", "")</f>
+        <v/>
+      </c>
+      <c r="F19" s="6">
+        <f>IF(OR(
+  AND(F18&gt;=90, COUNTIF($D$18:$Z$18, "&gt;=90")/COUNTA($D$18:$Z$18)&gt;0.05),
+  AND(F18&gt;=80,F18&lt;=89, (COUNTIF($D$18:$Z$18, "&gt;=80")-COUNTIF($D$18:$Z$18, "&gt;=90"))/COUNTA($D$18:$Z$18)&gt;0.2),
+  AND(F18&gt;=70,F18&lt;=79, (COUNTIF($D$18:$Z$18, "&gt;=70")-COUNTIF($D$18:$Z$18, "&gt;=80"))/COUNTA($D$18:$Z$18)&gt;0.4),
+  AND(F18&gt;=60,F18&lt;=69, (COUNTIF($D$18:$Z$18, "&gt;=60")-COUNTIF($D$18:$Z$18, "&gt;=70"))/COUNTA($D$18:$Z$18)&gt;0.3),
+  AND(F18&lt;=59, COUNTIF($D$18:$Z$18, "&lt;=59")/COUNTA($D$18:$Z$18)&gt;0.05)
+), "⚠ 超標！", "")</f>
+        <v/>
+      </c>
+      <c r="G19" s="6">
+        <f>IF(OR(
+  AND(G18&gt;=90, COUNTIF($D$18:$Z$18, "&gt;=90")/COUNTA($D$18:$Z$18)&gt;0.05),
+  AND(G18&gt;=80,G18&lt;=89, (COUNTIF($D$18:$Z$18, "&gt;=80")-COUNTIF($D$18:$Z$18, "&gt;=90"))/COUNTA($D$18:$Z$18)&gt;0.2),
+  AND(G18&gt;=70,G18&lt;=79, (COUNTIF($D$18:$Z$18, "&gt;=70")-COUNTIF($D$18:$Z$18, "&gt;=80"))/COUNTA($D$18:$Z$18)&gt;0.4),
+  AND(G18&gt;=60,G18&lt;=69, (COUNTIF($D$18:$Z$18, "&gt;=60")-COUNTIF($D$18:$Z$18, "&gt;=70"))/COUNTA($D$18:$Z$18)&gt;0.3),
+  AND(G18&lt;=59, COUNTIF($D$18:$Z$18, "&lt;=59")/COUNTA($D$18:$Z$18)&gt;0.05)
+), "⚠ 超標！", "")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="12">
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A2:I2"/>

</xml_diff>